<commit_message>
Se sube el nuevo archivo de salida.
</commit_message>
<xml_diff>
--- a/predicciones_finales.xlsx
+++ b/predicciones_finales.xlsx
@@ -829,7 +829,7 @@
         <v>27579</v>
       </c>
       <c r="B50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -901,7 +901,7 @@
         <v>27637</v>
       </c>
       <c r="B59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
@@ -1005,7 +1005,7 @@
         <v>27695</v>
       </c>
       <c r="B72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -1205,7 +1205,7 @@
         <v>27814</v>
       </c>
       <c r="B97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -1493,7 +1493,7 @@
         <v>28014</v>
       </c>
       <c r="B133" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="134">
@@ -1661,7 +1661,7 @@
         <v>28144</v>
       </c>
       <c r="B154" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="155">
@@ -1805,7 +1805,7 @@
         <v>28249</v>
       </c>
       <c r="B172" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="173">
@@ -1821,7 +1821,7 @@
         <v>28254</v>
       </c>
       <c r="B174" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="175">
@@ -2013,7 +2013,7 @@
         <v>28399</v>
       </c>
       <c r="B198" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="199">
@@ -2029,7 +2029,7 @@
         <v>28409</v>
       </c>
       <c r="B200" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="201">
@@ -2445,7 +2445,7 @@
         <v>28652</v>
       </c>
       <c r="B252" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="253">
@@ -3093,7 +3093,7 @@
         <v>28996</v>
       </c>
       <c r="B333" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="334">
@@ -3237,7 +3237,7 @@
         <v>29102</v>
       </c>
       <c r="B351" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="352">
@@ -3245,7 +3245,7 @@
         <v>29107</v>
       </c>
       <c r="B352" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="353">
@@ -3661,7 +3661,7 @@
         <v>29372</v>
       </c>
       <c r="B404" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="405">
@@ -3941,7 +3941,7 @@
         <v>29552</v>
       </c>
       <c r="B439" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="440">
@@ -4013,7 +4013,7 @@
         <v>29580</v>
       </c>
       <c r="B448" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="449">
@@ -4077,7 +4077,7 @@
         <v>29608</v>
       </c>
       <c r="B456" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="457">
@@ -4957,7 +4957,7 @@
         <v>30140</v>
       </c>
       <c r="B566" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="567">
@@ -5517,7 +5517,7 @@
         <v>30530</v>
       </c>
       <c r="B636" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="637">
@@ -6021,7 +6021,7 @@
         <v>30825</v>
       </c>
       <c r="B699" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="700">
@@ -6093,7 +6093,7 @@
         <v>30862</v>
       </c>
       <c r="B708" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="709">
@@ -6925,7 +6925,7 @@
         <v>31336</v>
       </c>
       <c r="B812" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="813">
@@ -7917,7 +7917,7 @@
         <v>31959</v>
       </c>
       <c r="B936" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="937">
@@ -8405,7 +8405,7 @@
         <v>32311</v>
       </c>
       <c r="B997" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="998">
@@ -8517,7 +8517,7 @@
         <v>32405</v>
       </c>
       <c r="B1011" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1012">
@@ -8869,7 +8869,7 @@
         <v>32658</v>
       </c>
       <c r="B1055" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1056">
@@ -8909,7 +8909,7 @@
         <v>32682</v>
       </c>
       <c r="B1060" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1061">
@@ -9373,7 +9373,7 @@
         <v>32995</v>
       </c>
       <c r="B1118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1119">
@@ -9477,7 +9477,7 @@
         <v>33057</v>
       </c>
       <c r="B1131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1132">
@@ -10509,7 +10509,7 @@
         <v>33793</v>
       </c>
       <c r="B1260" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1261">
@@ -10757,7 +10757,7 @@
         <v>33939</v>
       </c>
       <c r="B1291" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1292">
@@ -10981,7 +10981,7 @@
         <v>34095</v>
       </c>
       <c r="B1319" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1320">
@@ -11157,7 +11157,7 @@
         <v>34191</v>
       </c>
       <c r="B1341" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1342">
@@ -12157,7 +12157,7 @@
         <v>34767</v>
       </c>
       <c r="B1466" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1467">
@@ -12357,7 +12357,7 @@
         <v>34869</v>
       </c>
       <c r="B1491" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1492">
@@ -13349,7 +13349,7 @@
         <v>35443</v>
       </c>
       <c r="B1615" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1616">
@@ -13653,7 +13653,7 @@
         <v>35595</v>
       </c>
       <c r="B1653" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1654">
@@ -14053,7 +14053,7 @@
         <v>35868</v>
       </c>
       <c r="B1703" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1704">
@@ -14853,7 +14853,7 @@
         <v>36429</v>
       </c>
       <c r="B1803" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1804">
@@ -15621,7 +15621,7 @@
         <v>36951</v>
       </c>
       <c r="B1899" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1900">
@@ -16037,7 +16037,7 @@
         <v>37199</v>
       </c>
       <c r="B1951" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1952">
@@ -16309,7 +16309,7 @@
         <v>37317</v>
       </c>
       <c r="B1985" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1986">
@@ -16373,7 +16373,7 @@
         <v>37335</v>
       </c>
       <c r="B1993" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1994">
@@ -16429,7 +16429,7 @@
         <v>37359</v>
       </c>
       <c r="B2000" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2001">
@@ -16949,7 +16949,7 @@
         <v>37609</v>
       </c>
       <c r="B2065" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2066">
@@ -17333,7 +17333,7 @@
         <v>37832</v>
       </c>
       <c r="B2113" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2114">
@@ -17573,7 +17573,7 @@
         <v>38015</v>
       </c>
       <c r="B2143" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2144">
@@ -17661,7 +17661,7 @@
         <v>38098</v>
       </c>
       <c r="B2154" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2155">
@@ -17757,7 +17757,7 @@
         <v>38156</v>
       </c>
       <c r="B2166" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2167">
@@ -18133,7 +18133,7 @@
         <v>38355</v>
       </c>
       <c r="B2213" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2214">
@@ -18141,7 +18141,7 @@
         <v>38365</v>
       </c>
       <c r="B2214" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2215">
@@ -18613,7 +18613,7 @@
         <v>38664</v>
       </c>
       <c r="B2273" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2274">
@@ -19213,7 +19213,7 @@
         <v>39044</v>
       </c>
       <c r="B2348" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2349">
@@ -19773,7 +19773,7 @@
         <v>39444</v>
       </c>
       <c r="B2418" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2419">
@@ -19973,7 +19973,7 @@
         <v>39547</v>
       </c>
       <c r="B2443" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2444">
@@ -20181,7 +20181,7 @@
         <v>39687</v>
       </c>
       <c r="B2469" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2470">
@@ -20493,7 +20493,7 @@
         <v>39868</v>
       </c>
       <c r="B2508" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2509">
@@ -20525,7 +20525,7 @@
         <v>39891</v>
       </c>
       <c r="B2512" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2513">
@@ -21557,7 +21557,7 @@
         <v>40609</v>
       </c>
       <c r="B2641" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2642">
@@ -21909,7 +21909,7 @@
         <v>40806</v>
       </c>
       <c r="B2685" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2686">
@@ -21917,7 +21917,7 @@
         <v>40807</v>
       </c>
       <c r="B2686" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2687">
@@ -22285,7 +22285,7 @@
         <v>41098</v>
       </c>
       <c r="B2732" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2733">
@@ -22317,7 +22317,7 @@
         <v>41105</v>
       </c>
       <c r="B2736" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2737">
@@ -22325,7 +22325,7 @@
         <v>41106</v>
       </c>
       <c r="B2737" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2738">
@@ -22389,7 +22389,7 @@
         <v>41132</v>
       </c>
       <c r="B2745" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2746">
@@ -22877,7 +22877,7 @@
         <v>41443</v>
       </c>
       <c r="B2806" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2807">
@@ -22925,7 +22925,7 @@
         <v>41467</v>
       </c>
       <c r="B2812" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2813">
@@ -23141,7 +23141,7 @@
         <v>41576</v>
       </c>
       <c r="B2839" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2840">
@@ -23317,7 +23317,7 @@
         <v>41646</v>
       </c>
       <c r="B2861" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2862">
@@ -23421,7 +23421,7 @@
         <v>41709</v>
       </c>
       <c r="B2874" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2875">
@@ -23685,7 +23685,7 @@
         <v>41846</v>
       </c>
       <c r="B2907" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2908">
@@ -23749,7 +23749,7 @@
         <v>41900</v>
       </c>
       <c r="B2915" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2916">
@@ -24109,7 +24109,7 @@
         <v>42173</v>
       </c>
       <c r="B2960" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2961">
@@ -24181,7 +24181,7 @@
         <v>42218</v>
       </c>
       <c r="B2969" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2970">
@@ -24285,7 +24285,7 @@
         <v>42252</v>
       </c>
       <c r="B2982" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2983">
@@ -24373,7 +24373,7 @@
         <v>42293</v>
       </c>
       <c r="B2993" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2994">
@@ -24445,7 +24445,7 @@
         <v>42347</v>
       </c>
       <c r="B3002" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3003">
@@ -24525,7 +24525,7 @@
         <v>42411</v>
       </c>
       <c r="B3012" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3013">
@@ -25285,7 +25285,7 @@
         <v>42821</v>
       </c>
       <c r="B3107" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3108">
@@ -25325,7 +25325,7 @@
         <v>42843</v>
       </c>
       <c r="B3112" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3113">
@@ -25773,7 +25773,7 @@
         <v>43159</v>
       </c>
       <c r="B3168" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3169">
@@ -26021,7 +26021,7 @@
         <v>43277</v>
       </c>
       <c r="B3199" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3200">
@@ -26829,7 +26829,7 @@
         <v>43751</v>
       </c>
       <c r="B3300" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3301">
@@ -27677,7 +27677,7 @@
         <v>44294</v>
       </c>
       <c r="B3406" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3407">
@@ -27917,7 +27917,7 @@
         <v>44480</v>
       </c>
       <c r="B3436" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3437">
@@ -28269,7 +28269,7 @@
         <v>44686</v>
       </c>
       <c r="B3480" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3481">
@@ -28797,7 +28797,7 @@
         <v>45022</v>
       </c>
       <c r="B3546" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3547">
@@ -29141,7 +29141,7 @@
         <v>45208</v>
       </c>
       <c r="B3589" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3590">
@@ -31157,7 +31157,7 @@
         <v>46516</v>
       </c>
       <c r="B3841" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3842">
@@ -31997,7 +31997,7 @@
         <v>47007</v>
       </c>
       <c r="B3946" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3947">
@@ -32125,7 +32125,7 @@
         <v>47096</v>
       </c>
       <c r="B3962" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3963">
@@ -32141,7 +32141,7 @@
         <v>47133</v>
       </c>
       <c r="B3964" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3965">
@@ -32437,7 +32437,7 @@
         <v>47333</v>
       </c>
       <c r="B4001" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4002">
@@ -32461,7 +32461,7 @@
         <v>47336</v>
       </c>
       <c r="B4004" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4005">
@@ -32629,7 +32629,7 @@
         <v>47464</v>
       </c>
       <c r="B4025" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4026">
@@ -33317,7 +33317,7 @@
         <v>47827</v>
       </c>
       <c r="B4111" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4112">
@@ -33549,7 +33549,7 @@
         <v>47984</v>
       </c>
       <c r="B4140" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4141">
@@ -34357,7 +34357,7 @@
         <v>48496</v>
       </c>
       <c r="B4241" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4242">
@@ -34685,7 +34685,7 @@
         <v>48729</v>
       </c>
       <c r="B4282" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4283">
@@ -35189,7 +35189,7 @@
         <v>49024</v>
       </c>
       <c r="B4345" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4346">
@@ -35269,7 +35269,7 @@
         <v>49084</v>
       </c>
       <c r="B4355" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4356">
@@ -35581,7 +35581,7 @@
         <v>49297</v>
       </c>
       <c r="B4394" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4395">
@@ -35789,7 +35789,7 @@
         <v>49427</v>
       </c>
       <c r="B4420" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4421">
@@ -35981,7 +35981,7 @@
         <v>49524</v>
       </c>
       <c r="B4444" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4445">
@@ -36149,7 +36149,7 @@
         <v>49635</v>
       </c>
       <c r="B4465" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4466">
@@ -36205,7 +36205,7 @@
         <v>49691</v>
       </c>
       <c r="B4472" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4473">
@@ -36301,7 +36301,7 @@
         <v>49762</v>
       </c>
       <c r="B4484" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4485">
@@ -36389,7 +36389,7 @@
         <v>49823</v>
       </c>
       <c r="B4495" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4496">
@@ -36581,7 +36581,7 @@
         <v>49942</v>
       </c>
       <c r="B4519" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4520">
@@ -36709,7 +36709,7 @@
         <v>50013</v>
       </c>
       <c r="B4535" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4536">
@@ -37317,7 +37317,7 @@
         <v>50387</v>
       </c>
       <c r="B4611" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4612">
@@ -37413,7 +37413,7 @@
         <v>50432</v>
       </c>
       <c r="B4623" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4624">
@@ -37709,7 +37709,7 @@
         <v>50598</v>
       </c>
       <c r="B4660" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4661">
@@ -37749,7 +37749,7 @@
         <v>50616</v>
       </c>
       <c r="B4665" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4666">
@@ -37981,7 +37981,7 @@
         <v>50742</v>
       </c>
       <c r="B4694" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4695">
@@ -38061,7 +38061,7 @@
         <v>50799</v>
       </c>
       <c r="B4704" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4705">
@@ -38365,7 +38365,7 @@
         <v>50966</v>
       </c>
       <c r="B4742" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4743">
@@ -38453,7 +38453,7 @@
         <v>51009</v>
       </c>
       <c r="B4753" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4754">
@@ -38637,7 +38637,7 @@
         <v>51074</v>
       </c>
       <c r="B4776" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4777">
@@ -39341,7 +39341,7 @@
         <v>51495</v>
       </c>
       <c r="B4864" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4865">
@@ -39965,7 +39965,7 @@
         <v>51887</v>
       </c>
       <c r="B4942" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4943">
@@ -40021,7 +40021,7 @@
         <v>51928</v>
       </c>
       <c r="B4949" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4950">
@@ -40341,7 +40341,7 @@
         <v>52102</v>
       </c>
       <c r="B4989" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4990">
@@ -40365,7 +40365,7 @@
         <v>52114</v>
       </c>
       <c r="B4992" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4993">
@@ -40861,7 +40861,7 @@
         <v>52417</v>
       </c>
       <c r="B5054" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5055">
@@ -41349,7 +41349,7 @@
         <v>52727</v>
       </c>
       <c r="B5115" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5116">
@@ -42101,7 +42101,7 @@
         <v>53224</v>
       </c>
       <c r="B5209" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5210">
@@ -42573,7 +42573,7 @@
         <v>53565</v>
       </c>
       <c r="B5268" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5269">
@@ -42909,7 +42909,7 @@
         <v>53757</v>
       </c>
       <c r="B5310" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5311">
@@ -43109,7 +43109,7 @@
         <v>53868</v>
       </c>
       <c r="B5335" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5336">
@@ -43325,7 +43325,7 @@
         <v>53996</v>
       </c>
       <c r="B5362" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5363">
@@ -43421,7 +43421,7 @@
         <v>54060</v>
       </c>
       <c r="B5374" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5375">
@@ -44197,7 +44197,7 @@
         <v>54599</v>
       </c>
       <c r="B5471" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5472">
@@ -44469,7 +44469,7 @@
         <v>54782</v>
       </c>
       <c r="B5505" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5506">
@@ -44621,7 +44621,7 @@
         <v>54889</v>
       </c>
       <c r="B5524" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5525">
@@ -44741,7 +44741,7 @@
         <v>54936</v>
       </c>
       <c r="B5539" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5540">
@@ -44757,7 +44757,7 @@
         <v>54952</v>
       </c>
       <c r="B5541" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5542">
@@ -45245,7 +45245,7 @@
         <v>55244</v>
       </c>
       <c r="B5602" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5603">
@@ -45253,7 +45253,7 @@
         <v>55251</v>
       </c>
       <c r="B5603" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5604">
@@ -45877,7 +45877,7 @@
         <v>55632</v>
       </c>
       <c r="B5681" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5682">
@@ -45901,7 +45901,7 @@
         <v>55655</v>
       </c>
       <c r="B5684" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5685">

</xml_diff>